<commit_message>
9-12-25 todays code changes
</commit_message>
<xml_diff>
--- a/src/test/resources/ImportTemplate/Pushdown - Flat File-SQL.xlsx
+++ b/src/test/resources/ImportTemplate/Pushdown - Flat File-SQL.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Eclipse\ICEDQ\TestGenerator\src\test\resources\ImportTemplate\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C34AA40-46E2-44FD-A34E-8CBF56D2C289}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2521A989-6CA6-4649-829F-9FE32AE2EC89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -110,7 +110,7 @@
     <t>|</t>
   </si>
   <si>
-    <t>R001_FlatFile_SQL_Pushdown</t>
+    <t>R00_FlatFile-SQL_Pushdown</t>
   </si>
 </sst>
 </file>

</xml_diff>